<commit_message>
Updated distribution additions spreadsheet version
</commit_message>
<xml_diff>
--- a/team/models-and-sim-design/symbulate_distribution_additions.xlsx
+++ b/team/models-and-sim-design/symbulate_distribution_additions.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Distributions to Add" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Distributions to Add'!$A$1:$H$56</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Distributions to Add'!$A$1:$H$121</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="481">
   <si>
     <t xml:space="preserve">Distribution</t>
   </si>
@@ -232,6 +232,21 @@
     <t xml:space="preserve">Direct wrap; standard conjugate model for overdispersed binomial/count data</t>
   </si>
   <si>
+    <t xml:space="preserve">LKJ (correlation matrix prior)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multivariate (matrix-valued)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Bayesian Stats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bayesian Statistics, Multivariate Bayesian Modeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The default correlation-matrix prior in modern Bayesian workflows (Stan/PyMC); arguably as important as Wishart for this audience, and neither scipy nor Symbulate has it</t>
+  </si>
+  <si>
     <t xml:space="preserve">Generalized Pareto Distribution (GPD)</t>
   </si>
   <si>
@@ -292,9 +307,6 @@
     <t xml:space="preserve">Inverse Gamma</t>
   </si>
   <si>
-    <t xml:space="preserve">Statistics, Bayesian Stats</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bayesian Statistics</t>
   </si>
   <si>
@@ -400,6 +412,219 @@
     <t xml:space="preserve">Needs to operate generically over any existing discrete distribution (Poisson, Binomial, NegBinomial, Geometric) rather than being one class; a design decision, not a wrap</t>
   </si>
   <si>
+    <t xml:space="preserve">Beta-Pascal / Beta-Negative Binomial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actuarial Science, Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (betanbinom)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overdispersed negative-binomial counterpart to Beta-Binomial (already in this table); direct wrap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kumaraswamy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Engineering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Statistics, Simulation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beta look-alike with simple closed-form CDF/quantile; genuinely useful and easy to implement even without scipy backing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Management, Risk Analysis, Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulation, Risk Analysis, PERT Estimation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low-Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Special case of 4-parameter Beta; pairs directly with Triangular already in this table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Simulation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulation, Intro Statistics (CLT teaching)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean of n uniforms; companion to Irwin-Hall (sum vs. mean), useful CLT teaching pair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Irwin–Hall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (irwinhall)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum of n iid uniforms; should have been in the original table — genuine omission, not a low-priority call</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hyperexponential</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engineering, Operations Research</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Queueing Theory, Reliability Engineering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staple of queueing theory; models 'fast or slow' service-time heterogeneity via a mixture of exponentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hypoexponential</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Companion to Hyperexponential; models multi-stage service/failure processes as a sum of exponentials with distinct rates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-Gamma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loss Models, Extreme Value Theory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (loggamma)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mentioned in an earlier discussion of actuarial additions but never actually added — genuine omission being corrected here</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Truncated Normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Engineering, Bayesian Stats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Statistics, Bayesian Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (truncnorm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extremely common in practice; also shows the existing discrete-only truncation wrapper needs a continuous counterpart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scaled/Inverse Chi-Squared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (reparameterization of invgamma)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extremely common naming convention in Bayesian textbooks (e.g., Gelman et al.); worth a named alias even though mathematically = Inverse Gamma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gamma/Gompertz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gompertz mortality with Gamma frailty (population heterogeneity); natural extension once Gompertz/Makeham exist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exponentially Modified Gaussian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Psychology, Chemistry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Statistics, Psychometrics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (exponnorm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real applied use in chromatography and reaction-time modeling in psychology — broader audience than most lower-tier items</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skew t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finance, Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robust Statistics, Quantitative Finance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Natural extension of Skew-Normal already in this table; notable in finance/robust modeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reciprocal / Log-Uniform</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, ML, Engineering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Statistics, ML Hyperparameter Search</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (loguniform / reciprocal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mentioned in the very first response of this conversation and never actually added to the table — genuine omission being corrected here; also widely used for ML hyperparameter search ranges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotelling's T-squared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multivariate Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multivariate generalization of t²; pairs directly with Multivariate t already in this table, core topic in multivariate stats courses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categorical (formal Distribution-API version)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Univariate Discrete (non-numeric outcomes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intro Probability, ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No (not a scipy concept)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Directly closes the gap identified in the BoxModel vs. Empirical discussion — would give BoxModel-style non-numeric outcomes the same pmf/mode/plot access Empirical gives integer outcomes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General Mixture-Distribution Builder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modifier (any distribution)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial (component distributions exist; no generic container)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generic weighted-combination wrapper over any existing distributions; would also directly enable Hyperexponential as a special case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Continuous Truncation Wrapper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modifier (any continuous distribution)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial (truncnorm exists as one instance; no generic wrapper)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Continuous counterpart to the existing discrete truncation/zero-modification wrapper already in this table</t>
+  </si>
+  <si>
     <t xml:space="preserve">Negative Hypergeometric</t>
   </si>
   <si>
@@ -433,9 +658,6 @@
     <t xml:space="preserve">Simulation, Risk Modeling, Project Management</t>
   </si>
   <si>
-    <t xml:space="preserve">Simulation, Risk Analysis, PERT Estimation</t>
-  </si>
-  <si>
     <t xml:space="preserve">Yes (triang)</t>
   </si>
   <si>
@@ -460,9 +682,6 @@
     <t xml:space="preserve">Inverse Gaussian (Wald)</t>
   </si>
   <si>
-    <t xml:space="preserve">Statistics, Engineering</t>
-  </si>
-  <si>
     <t xml:space="preserve">Applied Statistics, Reliability</t>
   </si>
   <si>
@@ -496,18 +715,12 @@
     <t xml:space="preserve">Yes (gengamma)</t>
   </si>
   <si>
-    <t xml:space="preserve">Low-Medium</t>
-  </si>
-  <si>
     <t xml:space="preserve">scipy has it, but mapping parameters across its Gamma/Weibull/Exponential special cases needs care to present clearly to students</t>
   </si>
   <si>
     <t xml:space="preserve">Erlang</t>
   </si>
   <si>
-    <t xml:space="preserve">Engineering, Operations Research</t>
-  </si>
-  <si>
     <t xml:space="preserve">Queueing Theory</t>
   </si>
   <si>
@@ -568,6 +781,330 @@
     <t xml:space="preserve">Direct wrap; survival-analysis alternative to Weibull</t>
   </si>
   <si>
+    <t xml:space="preserve">Benford's Law</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Forensic Accounting, Data Science</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intro Stats, Forensic Accounting, Data Science Electives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classic fraud-detection/applied-stats teaching example; simple closed-form pmf P(d)=log10(1+1/d)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poisson Binomial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Data Science</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Statistics, Survey Sampling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum of independent non-identical Bernoullis; pmf needs convolution/recursive algorithm, not simply closed-form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zeta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Number Theory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Statistics, Power-Law Phenomena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (zipf)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infinite-support limiting case of Zipf; scipy's naming is a trap (zipf=zeta, zipfian=finite Zipf) worth flagging directly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noncentral Hypergeometric (Fisher's / Wallenius')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Genetics, Ecology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Statistics, Biostatistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (nchypergeom_fisher, nchypergeom_wallenius)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Models biased sampling without replacement; two related variants, some explanation needed to distinguish them</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Negative Multinomial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multivariate generalization of Negative Binomial, the way Multinomial generalizes Binomial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Degenerate / Point-Mass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intro Probability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trivial constant-outcome distribution; useful building block for mixtures and edge-case teaching</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Birthday Distribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Univariate Discrete (combinatorial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intro Probability, Combinatorics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classic 'birthday problem' teaching distribution; likely more valuable as a worked example than a formal class</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coupon Collector Distribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classic combinatorial waiting-time problem; pairs pedagogically with Birthday Distribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arcsine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Probability Theory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probability Theory, Random Walks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (arcsine)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beta(1/2,1/2) special case; appears in random walk / order statistics theory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mathematical Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (chi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Square root of Chi-square; parent distribution of Rayleigh and Maxwell-Boltzmann</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noncentral Beta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power Analysis (R²/partial correlation tests)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed absent from scipy; used in power analysis for R² and partial-correlation tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exponential Power / Generalized Normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Signal Processing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (exponpow, gennorm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unifies Normal/Laplace/Uniform-like tail behavior via one shape parameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beta Prime / Inverted Beta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mathematical Statistics, Bayesian Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (betaprime)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Related to F-distribution; used in Bayesian variance modeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power / Power-Function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Reliability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (powerlaw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beta(a,1) special case; simple but distinct named distribution worth surfacing directly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two-Sided Power (TSP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulation, Risk Analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generalizes Triangular the way GEV generalizes Gumbel; natural extension once Triangular exists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generalized Beta of the Second Kind (GB2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loss Models, Income Distribution Modeling (grad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4-parameter umbrella family over Burr/Singh-Maddala/Lomax already in this table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dagum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Income Distribution Modeling, Loss Models</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Income-distribution family sitting alongside Burr/Singh-Maddala already in this table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Folded-Normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (foldnorm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">|X| where X~Normal(μ,σ) with μ≠0; distinct from Half-Normal already in this table, which assumes μ=0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maxwell-Boltzmann</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Physics, Engineering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistical Mechanics, Physics-Stats Crossover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (maxwell)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classic physics speed distribution; special case of Chi with 3 degrees of freedom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wigner Semicircle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Physics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Random Matrix Theory (grad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (semicircular)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foundational random matrix theory result; notable for grad-level probability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trapezoidal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (trapezoid)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generalizes Triangular/Uniform; common in simulation modeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generalized Logistic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Statistics, Extreme Value Theory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (genlogistic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skewed generalization of Logistic already in this table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marshall–Olkin Exponential</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Univariate Continuous (bivariate construction)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engineering, Reliability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reliability Engineering (grad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Models dependent component failure times via a shock-model construction; notable in reliability engineering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Continuous Bernoulli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Machine Learning, Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ML/Data Science</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modern ML use (VAE probabilistic pixel outputs); relevant for ML-adjacent stats courses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logit-Normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bayesian Statistics, ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Common for modeling probabilities in Bayesian/ML contexts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">von Mises–Fisher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multivariate (directional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Directional/Circular Statistics (grad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (vonmises_fisher)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spherical generalization of Von Mises already in this table, to higher dimensions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order Statistics / Finite Order Statistic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modifier/Feature (derived from any distribution)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No (not a distribution per se)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribution of the k-th order statistic of n iid draws; likely already achievable via existing RV transformations in Symbulate — worth confirming before building anything new</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test-Statistic Sampling Distributions (KS, Kolmogorov, Anderson-Darling)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Univariate Continuous (special-purpose)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mathematical Statistics, Goodness-of-Fit Testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (ksone, kstwobign, kstwo, anderson)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A different category from modeling distributions — these are sampling distributions of goodness-of-fit test statistics; direct scipy wraps</t>
+  </si>
+  <si>
     <t xml:space="preserve">Von Mises</t>
   </si>
   <si>
@@ -676,9 +1213,6 @@
     <t xml:space="preserve">Stable (Lévy-stable)</t>
   </si>
   <si>
-    <t xml:space="preserve">Finance, Statistics</t>
-  </si>
-  <si>
     <t xml:space="preserve">Quantitative Finance, Probability Theory (grad)</t>
   </si>
   <si>
@@ -779,6 +1313,159 @@
   </si>
   <si>
     <t xml:space="preserve">Not in scipy, but has a known closed-form CDF, so custom implementation is straightforward even though not a wrap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rademacher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probability Theory, Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trivial variant of Bernoulli (±1, p=.5); useful in random-sign/Monte Carlo contexts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zipf-Mandelbrot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics, Linguistics, Information Theory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Statistics, NLP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generalizes Zipf with an added parameter; needs custom normalizing-constant computation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discrete ArcSine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Random Walks, Stochastic Processes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discrete counterpart to continuous Arcsine; pmf derived from random-walk sign-change theory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boltzmann</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Physics, Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistical-physics distribution over discrete energy levels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Borel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probability Theory, Operations Research</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branching Processes, Queueing Theory (grad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arises from branching processes and busy-period queueing analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matching Distribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classic derangement/matching problem distribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noncentral Chi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mathematical Statistics, Signal Processing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Less common than noncentral chi-square, but a real remaining gap once that one is added</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doubly Noncentral t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advanced Mathematical Statistics (grad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both numerator and denominator noncentral; no standard package support, advanced power-analysis edge case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doubly Noncentral F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same rationale as Doubly Noncentral t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hyperbolic-Secant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (hypsecant)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logistic-like shape; occasional alternative to Normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marchenko–Pastur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pairs with Wigner Semicircle in random matrix theory; density is piecewise depending on aspect-ratio parameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracy–Widom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same cluster as Semicircle/Marchenko-Pastur; no closed-form density, defined via Painlevé differential equations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U-Quadratic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bathtub-shaped density on a bounded interval; niche but simple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fisher's z-distribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mathematical Statistics (historical/classical)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classical transform of F; historically important but rarely used directly today</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hyperbolic (general family)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umbrella family for NIG and Variance-Gamma already in this table; the general family is harder to implement than its special cases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voigt Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spectroscopy, Signal Processing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (voigt_profile)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Convolution of Normal+Cauchy; used in spectroscopy and engineering signal analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wakeby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hydrology, Environmental Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Environmental/Hydrology Statistics (grad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flood-frequency modeling; 5-parameter family with no simple closed-form density, defined via quantile function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matrix t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matrix-variate generalization, natural companion to Matrix Normal already in this table; grad-level</t>
   </si>
 </sst>
 </file>
@@ -1255,17 +1942,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1450,7 +2136,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>40</v>
       </c>
@@ -1528,7 +2214,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>56</v>
       </c>
@@ -1606,85 +2292,85 @@
         <v>68</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
         <v>69</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>9</v>
+        <v>70</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="E14" s="4" t="s">
         <v>72</v>
       </c>
+      <c r="E14" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="F14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" s="2" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="B15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>76</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>81</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>14</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>84</v>
       </c>
@@ -1692,39 +2378,39 @@
         <v>9</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>90</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>91</v>
@@ -1744,103 +2430,103 @@
         <v>9</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="D21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E21" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="F21" s="2" t="s">
+      <c r="G21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H21" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="G21" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H21" s="2" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>105</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>106</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
         <v>108</v>
       </c>
@@ -1848,884 +2534,2574 @@
         <v>41</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>35</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>112</v>
+        <v>71</v>
       </c>
       <c r="D24" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="E24" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="F24" s="2" t="s">
+      <c r="G24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H24" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="D25" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="E26" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>123</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
         <v>125</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>64</v>
+        <v>126</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>126</v>
+        <v>27</v>
       </c>
       <c r="D27" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="G27" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F28" s="2" t="s">
+      <c r="G28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="E29" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H29" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="E29" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F29" s="2" t="s">
+    </row>
+    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H29" s="2" t="s">
+      <c r="B30" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C30" s="2" t="s">
+      <c r="E30" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="H30" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="E30" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F30" s="2" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="G30" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H30" s="2" t="s">
+      <c r="B31" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
+      <c r="D31" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C31" s="2" t="s">
+      <c r="E31" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D31" s="2" t="s">
+    </row>
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="E31" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F31" s="2" t="s">
+      <c r="B32" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="G31" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H31" s="2" t="s">
+      <c r="G32" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="B33" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D33" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="E32" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F32" s="2" t="s">
+      <c r="E33" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H33" s="2" t="s">
         <v>152</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>128</v>
+        <v>151</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>77</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>162</v>
+        <v>34</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="D35" s="2" t="s">
+      <c r="B37" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F37" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="E35" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F35" s="2" t="s">
+      <c r="G37" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H37" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="G35" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H35" s="2" t="s">
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
+      <c r="B38" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H38" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="D39" s="2" t="s">
+      <c r="G41" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H41" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="E39" s="6" t="s">
+    </row>
+    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="F39" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2" t="s">
-        <v>195</v>
-      </c>
       <c r="B42" s="2" t="s">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>77</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>34</v>
       </c>
       <c r="G42" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E43" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="H42" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>183</v>
-      </c>
       <c r="F43" s="2" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>64</v>
+        <v>193</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>145</v>
+        <v>71</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>183</v>
+        <v>161</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>77</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>34</v>
+        <v>194</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>35</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H46" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H45" s="2" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="H46" s="2" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>183</v>
+        <v>202</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>203</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>157</v>
+        <v>30</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F49" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C48" s="2" t="s">
+      <c r="G49" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H49" s="2" t="s">
         <v>217</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H48" s="2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D50" s="2" t="s">
+      <c r="E51" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F51" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="E50" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F50" s="2" t="s">
+      <c r="G51" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H51" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="G50" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H50" s="2" t="s">
+    </row>
+    <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="2" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="51" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="2" t="s">
+      <c r="B52" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="E52" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="C51" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="D51" s="2" t="s">
+      <c r="G52" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H52" s="2" t="s">
         <v>230</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="H51" s="2" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="H52" s="2" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H53" s="2" t="s">
         <v>234</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H54" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B54" s="2" t="s">
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="B55" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C55" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="D54" s="2" t="s">
+      <c r="D55" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F55" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="E54" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="H54" s="2" t="s">
+      <c r="G55" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H55" s="2" t="s">
         <v>242</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="H55" s="2" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C56" s="2" t="s">
+      <c r="B57" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="D56" s="2" t="s">
+      <c r="E57" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F57" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="E56" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F56" s="2" t="s">
+      <c r="G57" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F58" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G56" s="2" t="s">
+      <c r="G58" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G59" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H56" s="2" t="s">
-        <v>251</v>
+      <c r="H59" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E63" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="E64" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H75" s="2" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H76" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H77" s="2" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="E78" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H78" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="E79" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H79" s="2" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E80" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="E81" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H81" s="2" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="E82" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E83" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H83" s="2" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="E84" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="E85" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H85" s="2" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="E86" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H86" s="2" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="E87" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H87" s="2" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="E88" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="G88" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H88" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G89" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H89" s="2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="E90" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="G90" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H90" s="2" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G91" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H91" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H92" s="2" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G93" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H93" s="2" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="G94" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H94" s="2" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="E95" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="G95" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H95" s="2" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E96" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H96" s="2" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="E97" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="G97" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H97" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="E98" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G98" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H98" s="2" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G99" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H99" s="2" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E100" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H100" s="2" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E101" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G101" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H101" s="2" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="E102" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G102" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H102" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="E103" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G103" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H103" s="2" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E104" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G104" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H104" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="E105" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G105" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H105" s="2" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="E106" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G106" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H106" s="2" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="E107" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F107" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G107" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H107" s="2" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="E108" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F108" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G108" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H108" s="2" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="E109" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F109" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G109" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H109" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="E110" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F110" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G110" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H110" s="2" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="E111" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F111" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G111" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H111" s="2" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="E112" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F112" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G112" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H112" s="2" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E113" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="G113" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H113" s="2" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="E114" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H114" s="2" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="E115" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F115" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G115" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H115" s="2" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E116" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F116" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G116" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H116" s="2" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="E117" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F117" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G117" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H117" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E118" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G118" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H118" s="2" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="E119" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="G119" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H119" s="2" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="E120" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G120" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H120" s="2" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E121" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F121" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H121" s="2" t="s">
+        <v>480</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H56"/>
+  <autoFilter ref="A1:H121"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>